<commit_message>
Live event registrations from PheedLoop
Adds the pheedloop-sync Edge Function (hourly via pg_cron), shows live
registrations in the Engagement section, and makes registrations optional
on the template's Events tab.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HBvLiZRp3wB8j46GxyLbc4
</commit_message>
<xml_diff>
--- a/template/MCE-monthly-data-template.xlsx
+++ b/template/MCE-monthly-data-template.xlsx
@@ -222,12 +222,17 @@
   <commentList>
     <comment ref="A4" authorId="0" shapeId="0">
       <text>
-        <t>Short unique code you'll reuse every month, e.g. CN2026, CAIC2027</t>
+        <t>The event's code in PheedLoop (in the event URL or Event Settings)</t>
+      </text>
+    </comment>
+    <comment ref="B4" authorId="0" shapeId="0">
+      <text>
+        <t>Optional for PheedLoop events</t>
       </text>
     </comment>
     <comment ref="C4" authorId="0" shapeId="0">
       <text>
-        <t>YYYY-MM-DD</t>
+        <t>YYYY-MM-DD, optional for PheedLoop events</t>
       </text>
     </comment>
     <comment ref="D4" authorId="0" shapeId="0">
@@ -243,6 +248,11 @@
     <comment ref="H4" authorId="0" shapeId="0">
       <text>
         <t>Optional, links this event to last year's for comparison</t>
+      </text>
+    </comment>
+    <comment ref="I4" authorId="0" shapeId="0">
+      <text>
+        <t>Leave blank: PheedLoop fills this in</t>
       </text>
     </comment>
     <comment ref="J4" authorId="0" shapeId="0">
@@ -706,7 +716,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>PheedLoop → each event's registration report as of the last day of the month.</t>
+          <t>Registrations update automatically from PheedLoop. Add targets, revenue to date and last year's event code on the Events tab.</t>
         </is>
       </c>
     </row>
@@ -2957,7 +2967,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>One row per event that was open for registration during the month. Registrations and revenue are totals to date on the last day of the month.</t>
+          <t>Registrations come from PheedLoop automatically every hour. Use this tab only to add targets, revenue to date and last year's event code. Only the event code is required.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Template: prefill Events tab with current PheedLoop events
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HBvLiZRp3wB8j46GxyLbc4
</commit_message>
<xml_diff>
--- a/template/MCE-monthly-data-template.xlsx
+++ b/template/MCE-monthly-data-template.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +69,13 @@
       <color rgb="000000FF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001B2A5A"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -90,6 +95,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E8ECF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF1F6"/>
       </patternFill>
     </fill>
   </fills>
@@ -119,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -135,9 +145,11 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2971,6 +2983,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Rows below are your current PheedLoop events. Add targets, revenue and last year's code in the yellow cells; delete rows you don't need.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -3029,393 +3048,483 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="n"/>
-      <c r="B5" s="13" t="n"/>
-      <c r="C5" s="14" t="n"/>
-      <c r="D5" s="14" t="n"/>
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>EVELJKYPBEJHY</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Canada Night 2026</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>46329</v>
+      </c>
+      <c r="D5" s="15" t="n"/>
       <c r="E5" s="11" t="n"/>
       <c r="F5" s="11" t="n"/>
-      <c r="G5" s="15" t="n"/>
-      <c r="H5" s="13" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="17" t="n"/>
       <c r="I5" s="11" t="n"/>
-      <c r="J5" s="15" t="n"/>
+      <c r="J5" s="16" t="n"/>
       <c r="K5" s="11" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="n"/>
-      <c r="B6" s="13" t="n"/>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="14" t="n"/>
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>EVEBXNZTBEUUH</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Student Automotive Innovation Challenge 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>46344</v>
+      </c>
+      <c r="D6" s="15" t="n"/>
       <c r="E6" s="11" t="n"/>
       <c r="F6" s="11" t="n"/>
-      <c r="G6" s="15" t="n"/>
-      <c r="H6" s="13" t="n"/>
+      <c r="G6" s="16" t="n"/>
+      <c r="H6" s="17" t="n"/>
       <c r="I6" s="11" t="n"/>
-      <c r="J6" s="15" t="n"/>
+      <c r="J6" s="16" t="n"/>
       <c r="K6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="n"/>
-      <c r="B7" s="13" t="n"/>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="14" t="n"/>
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>EVEAQFBMZWRVS</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>YPA Community Learning and Leadership Social 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>46359</v>
+      </c>
+      <c r="D7" s="15" t="n"/>
       <c r="E7" s="11" t="n"/>
       <c r="F7" s="11" t="n"/>
-      <c r="G7" s="15" t="n"/>
-      <c r="H7" s="13" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="17" t="n"/>
       <c r="I7" s="11" t="n"/>
-      <c r="J7" s="15" t="n"/>
+      <c r="J7" s="16" t="n"/>
       <c r="K7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="n"/>
-      <c r="B8" s="13" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>EVEMZGBXYIECC</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>AIA Canada Manitoba Division Holiday Luncheon 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>46367</v>
+      </c>
+      <c r="D8" s="15" t="n"/>
       <c r="E8" s="11" t="n"/>
       <c r="F8" s="11" t="n"/>
-      <c r="G8" s="15" t="n"/>
-      <c r="H8" s="13" t="n"/>
+      <c r="G8" s="16" t="n"/>
+      <c r="H8" s="17" t="n"/>
       <c r="I8" s="11" t="n"/>
-      <c r="J8" s="15" t="n"/>
+      <c r="J8" s="16" t="n"/>
       <c r="K8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="n"/>
-      <c r="B9" s="13" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>EVEHLZEOSVFCO</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>CAIC 2027</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>46476</v>
+      </c>
+      <c r="D9" s="15" t="n"/>
       <c r="E9" s="11" t="n"/>
       <c r="F9" s="11" t="n"/>
-      <c r="G9" s="15" t="n"/>
-      <c r="H9" s="13" t="n"/>
+      <c r="G9" s="16" t="n"/>
+      <c r="H9" s="17" t="n"/>
       <c r="I9" s="11" t="n"/>
-      <c r="J9" s="15" t="n"/>
+      <c r="J9" s="16" t="n"/>
       <c r="K9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="n"/>
-      <c r="B10" s="13" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="14" t="n"/>
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>EVERJBXTUBTOJ</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>CCIF Montreal 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D10" s="15" t="n"/>
       <c r="E10" s="11" t="n"/>
       <c r="F10" s="11" t="n"/>
-      <c r="G10" s="15" t="n"/>
-      <c r="H10" s="13" t="n"/>
+      <c r="G10" s="16" t="n"/>
+      <c r="H10" s="17" t="n"/>
       <c r="I10" s="11" t="n"/>
-      <c r="J10" s="15" t="n"/>
+      <c r="J10" s="16" t="n"/>
       <c r="K10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="n"/>
-      <c r="B11" s="13" t="n"/>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="14" t="n"/>
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>EVEYTSAMYGMAZ</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Tournoi de golf de la division du Québec de l'AIA Canada 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D11" s="15" t="n"/>
       <c r="E11" s="11" t="n"/>
       <c r="F11" s="11" t="n"/>
-      <c r="G11" s="15" t="n"/>
-      <c r="H11" s="13" t="n"/>
+      <c r="G11" s="16" t="n"/>
+      <c r="H11" s="17" t="n"/>
       <c r="I11" s="11" t="n"/>
-      <c r="J11" s="15" t="n"/>
+      <c r="J11" s="16" t="n"/>
       <c r="K11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="n"/>
-      <c r="B12" s="13" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="14" t="n"/>
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>EVESVVXRAORUS</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>AIA Canada Alberta Division golf tournament 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D12" s="15" t="n"/>
       <c r="E12" s="11" t="n"/>
       <c r="F12" s="11" t="n"/>
-      <c r="G12" s="15" t="n"/>
-      <c r="H12" s="13" t="n"/>
+      <c r="G12" s="16" t="n"/>
+      <c r="H12" s="17" t="n"/>
       <c r="I12" s="11" t="n"/>
-      <c r="J12" s="15" t="n"/>
+      <c r="J12" s="16" t="n"/>
       <c r="K12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="n"/>
-      <c r="B13" s="13" t="n"/>
-      <c r="C13" s="14" t="n"/>
-      <c r="D13" s="14" t="n"/>
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>EVEEACRKBFWWT</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>AIA Canada Manitoba Division golf tournament 2026</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="n">
+        <v>46268</v>
+      </c>
+      <c r="D13" s="15" t="n"/>
       <c r="E13" s="11" t="n"/>
       <c r="F13" s="11" t="n"/>
-      <c r="G13" s="15" t="n"/>
-      <c r="H13" s="13" t="n"/>
+      <c r="G13" s="16" t="n"/>
+      <c r="H13" s="17" t="n"/>
       <c r="I13" s="11" t="n"/>
-      <c r="J13" s="15" t="n"/>
+      <c r="J13" s="16" t="n"/>
       <c r="K13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="n"/>
-      <c r="B14" s="13" t="n"/>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="14" t="n"/>
+      <c r="A14" s="17" t="n"/>
+      <c r="B14" s="17" t="n"/>
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="15" t="n"/>
       <c r="E14" s="11" t="n"/>
       <c r="F14" s="11" t="n"/>
-      <c r="G14" s="15" t="n"/>
-      <c r="H14" s="13" t="n"/>
+      <c r="G14" s="16" t="n"/>
+      <c r="H14" s="17" t="n"/>
       <c r="I14" s="11" t="n"/>
-      <c r="J14" s="15" t="n"/>
+      <c r="J14" s="16" t="n"/>
       <c r="K14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="n"/>
-      <c r="B15" s="13" t="n"/>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="14" t="n"/>
+      <c r="A15" s="17" t="n"/>
+      <c r="B15" s="17" t="n"/>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="15" t="n"/>
       <c r="E15" s="11" t="n"/>
       <c r="F15" s="11" t="n"/>
-      <c r="G15" s="15" t="n"/>
-      <c r="H15" s="13" t="n"/>
+      <c r="G15" s="16" t="n"/>
+      <c r="H15" s="17" t="n"/>
       <c r="I15" s="11" t="n"/>
-      <c r="J15" s="15" t="n"/>
+      <c r="J15" s="16" t="n"/>
       <c r="K15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="n"/>
-      <c r="B16" s="13" t="n"/>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="14" t="n"/>
+      <c r="A16" s="17" t="n"/>
+      <c r="B16" s="17" t="n"/>
+      <c r="C16" s="15" t="n"/>
+      <c r="D16" s="15" t="n"/>
       <c r="E16" s="11" t="n"/>
       <c r="F16" s="11" t="n"/>
-      <c r="G16" s="15" t="n"/>
-      <c r="H16" s="13" t="n"/>
+      <c r="G16" s="16" t="n"/>
+      <c r="H16" s="17" t="n"/>
       <c r="I16" s="11" t="n"/>
-      <c r="J16" s="15" t="n"/>
+      <c r="J16" s="16" t="n"/>
       <c r="K16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="n"/>
-      <c r="B17" s="13" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="14" t="n"/>
+      <c r="A17" s="17" t="n"/>
+      <c r="B17" s="17" t="n"/>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="15" t="n"/>
       <c r="E17" s="11" t="n"/>
       <c r="F17" s="11" t="n"/>
-      <c r="G17" s="15" t="n"/>
-      <c r="H17" s="13" t="n"/>
+      <c r="G17" s="16" t="n"/>
+      <c r="H17" s="17" t="n"/>
       <c r="I17" s="11" t="n"/>
-      <c r="J17" s="15" t="n"/>
+      <c r="J17" s="16" t="n"/>
       <c r="K17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="n"/>
-      <c r="B18" s="13" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="14" t="n"/>
+      <c r="A18" s="17" t="n"/>
+      <c r="B18" s="17" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="15" t="n"/>
       <c r="E18" s="11" t="n"/>
       <c r="F18" s="11" t="n"/>
-      <c r="G18" s="15" t="n"/>
-      <c r="H18" s="13" t="n"/>
+      <c r="G18" s="16" t="n"/>
+      <c r="H18" s="17" t="n"/>
       <c r="I18" s="11" t="n"/>
-      <c r="J18" s="15" t="n"/>
+      <c r="J18" s="16" t="n"/>
       <c r="K18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="n"/>
-      <c r="B19" s="13" t="n"/>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="14" t="n"/>
+      <c r="A19" s="17" t="n"/>
+      <c r="B19" s="17" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
       <c r="E19" s="11" t="n"/>
       <c r="F19" s="11" t="n"/>
-      <c r="G19" s="15" t="n"/>
-      <c r="H19" s="13" t="n"/>
+      <c r="G19" s="16" t="n"/>
+      <c r="H19" s="17" t="n"/>
       <c r="I19" s="11" t="n"/>
-      <c r="J19" s="15" t="n"/>
+      <c r="J19" s="16" t="n"/>
       <c r="K19" s="11" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="n"/>
-      <c r="B20" s="13" t="n"/>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="14" t="n"/>
+      <c r="A20" s="17" t="n"/>
+      <c r="B20" s="17" t="n"/>
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="15" t="n"/>
       <c r="E20" s="11" t="n"/>
       <c r="F20" s="11" t="n"/>
-      <c r="G20" s="15" t="n"/>
-      <c r="H20" s="13" t="n"/>
+      <c r="G20" s="16" t="n"/>
+      <c r="H20" s="17" t="n"/>
       <c r="I20" s="11" t="n"/>
-      <c r="J20" s="15" t="n"/>
+      <c r="J20" s="16" t="n"/>
       <c r="K20" s="11" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="n"/>
-      <c r="B21" s="13" t="n"/>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="14" t="n"/>
+      <c r="A21" s="17" t="n"/>
+      <c r="B21" s="17" t="n"/>
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="15" t="n"/>
       <c r="E21" s="11" t="n"/>
       <c r="F21" s="11" t="n"/>
-      <c r="G21" s="15" t="n"/>
-      <c r="H21" s="13" t="n"/>
+      <c r="G21" s="16" t="n"/>
+      <c r="H21" s="17" t="n"/>
       <c r="I21" s="11" t="n"/>
-      <c r="J21" s="15" t="n"/>
+      <c r="J21" s="16" t="n"/>
       <c r="K21" s="11" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="n"/>
-      <c r="B22" s="13" t="n"/>
-      <c r="C22" s="14" t="n"/>
-      <c r="D22" s="14" t="n"/>
+      <c r="A22" s="17" t="n"/>
+      <c r="B22" s="17" t="n"/>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="15" t="n"/>
       <c r="E22" s="11" t="n"/>
       <c r="F22" s="11" t="n"/>
-      <c r="G22" s="15" t="n"/>
-      <c r="H22" s="13" t="n"/>
+      <c r="G22" s="16" t="n"/>
+      <c r="H22" s="17" t="n"/>
       <c r="I22" s="11" t="n"/>
-      <c r="J22" s="15" t="n"/>
+      <c r="J22" s="16" t="n"/>
       <c r="K22" s="11" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="n"/>
-      <c r="B23" s="13" t="n"/>
-      <c r="C23" s="14" t="n"/>
-      <c r="D23" s="14" t="n"/>
+      <c r="A23" s="17" t="n"/>
+      <c r="B23" s="17" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
       <c r="E23" s="11" t="n"/>
       <c r="F23" s="11" t="n"/>
-      <c r="G23" s="15" t="n"/>
-      <c r="H23" s="13" t="n"/>
+      <c r="G23" s="16" t="n"/>
+      <c r="H23" s="17" t="n"/>
       <c r="I23" s="11" t="n"/>
-      <c r="J23" s="15" t="n"/>
+      <c r="J23" s="16" t="n"/>
       <c r="K23" s="11" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="n"/>
-      <c r="B24" s="13" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="14" t="n"/>
+      <c r="A24" s="17" t="n"/>
+      <c r="B24" s="17" t="n"/>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="15" t="n"/>
       <c r="E24" s="11" t="n"/>
       <c r="F24" s="11" t="n"/>
-      <c r="G24" s="15" t="n"/>
-      <c r="H24" s="13" t="n"/>
+      <c r="G24" s="16" t="n"/>
+      <c r="H24" s="17" t="n"/>
       <c r="I24" s="11" t="n"/>
-      <c r="J24" s="15" t="n"/>
+      <c r="J24" s="16" t="n"/>
       <c r="K24" s="11" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="n"/>
-      <c r="B25" s="13" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="14" t="n"/>
+      <c r="A25" s="17" t="n"/>
+      <c r="B25" s="17" t="n"/>
+      <c r="C25" s="15" t="n"/>
+      <c r="D25" s="15" t="n"/>
       <c r="E25" s="11" t="n"/>
       <c r="F25" s="11" t="n"/>
-      <c r="G25" s="15" t="n"/>
-      <c r="H25" s="13" t="n"/>
+      <c r="G25" s="16" t="n"/>
+      <c r="H25" s="17" t="n"/>
       <c r="I25" s="11" t="n"/>
-      <c r="J25" s="15" t="n"/>
+      <c r="J25" s="16" t="n"/>
       <c r="K25" s="11" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="n"/>
-      <c r="B26" s="13" t="n"/>
-      <c r="C26" s="14" t="n"/>
-      <c r="D26" s="14" t="n"/>
+      <c r="A26" s="17" t="n"/>
+      <c r="B26" s="17" t="n"/>
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="15" t="n"/>
       <c r="E26" s="11" t="n"/>
       <c r="F26" s="11" t="n"/>
-      <c r="G26" s="15" t="n"/>
-      <c r="H26" s="13" t="n"/>
+      <c r="G26" s="16" t="n"/>
+      <c r="H26" s="17" t="n"/>
       <c r="I26" s="11" t="n"/>
-      <c r="J26" s="15" t="n"/>
+      <c r="J26" s="16" t="n"/>
       <c r="K26" s="11" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="n"/>
-      <c r="B27" s="13" t="n"/>
-      <c r="C27" s="14" t="n"/>
-      <c r="D27" s="14" t="n"/>
+      <c r="A27" s="17" t="n"/>
+      <c r="B27" s="17" t="n"/>
+      <c r="C27" s="15" t="n"/>
+      <c r="D27" s="15" t="n"/>
       <c r="E27" s="11" t="n"/>
       <c r="F27" s="11" t="n"/>
-      <c r="G27" s="15" t="n"/>
-      <c r="H27" s="13" t="n"/>
+      <c r="G27" s="16" t="n"/>
+      <c r="H27" s="17" t="n"/>
       <c r="I27" s="11" t="n"/>
-      <c r="J27" s="15" t="n"/>
+      <c r="J27" s="16" t="n"/>
       <c r="K27" s="11" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="n"/>
-      <c r="B28" s="13" t="n"/>
-      <c r="C28" s="14" t="n"/>
-      <c r="D28" s="14" t="n"/>
+      <c r="A28" s="17" t="n"/>
+      <c r="B28" s="17" t="n"/>
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="15" t="n"/>
       <c r="E28" s="11" t="n"/>
       <c r="F28" s="11" t="n"/>
-      <c r="G28" s="15" t="n"/>
-      <c r="H28" s="13" t="n"/>
+      <c r="G28" s="16" t="n"/>
+      <c r="H28" s="17" t="n"/>
       <c r="I28" s="11" t="n"/>
-      <c r="J28" s="15" t="n"/>
+      <c r="J28" s="16" t="n"/>
       <c r="K28" s="11" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="n"/>
-      <c r="B29" s="13" t="n"/>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="14" t="n"/>
+      <c r="A29" s="17" t="n"/>
+      <c r="B29" s="17" t="n"/>
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="15" t="n"/>
       <c r="E29" s="11" t="n"/>
       <c r="F29" s="11" t="n"/>
-      <c r="G29" s="15" t="n"/>
-      <c r="H29" s="13" t="n"/>
+      <c r="G29" s="16" t="n"/>
+      <c r="H29" s="17" t="n"/>
       <c r="I29" s="11" t="n"/>
-      <c r="J29" s="15" t="n"/>
+      <c r="J29" s="16" t="n"/>
       <c r="K29" s="11" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="n"/>
-      <c r="B30" s="13" t="n"/>
-      <c r="C30" s="14" t="n"/>
-      <c r="D30" s="14" t="n"/>
+      <c r="A30" s="17" t="n"/>
+      <c r="B30" s="17" t="n"/>
+      <c r="C30" s="15" t="n"/>
+      <c r="D30" s="15" t="n"/>
       <c r="E30" s="11" t="n"/>
       <c r="F30" s="11" t="n"/>
-      <c r="G30" s="15" t="n"/>
-      <c r="H30" s="13" t="n"/>
+      <c r="G30" s="16" t="n"/>
+      <c r="H30" s="17" t="n"/>
       <c r="I30" s="11" t="n"/>
-      <c r="J30" s="15" t="n"/>
+      <c r="J30" s="16" t="n"/>
       <c r="K30" s="11" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="n"/>
-      <c r="B31" s="13" t="n"/>
-      <c r="C31" s="14" t="n"/>
-      <c r="D31" s="14" t="n"/>
+      <c r="A31" s="17" t="n"/>
+      <c r="B31" s="17" t="n"/>
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="15" t="n"/>
       <c r="E31" s="11" t="n"/>
       <c r="F31" s="11" t="n"/>
-      <c r="G31" s="15" t="n"/>
-      <c r="H31" s="13" t="n"/>
+      <c r="G31" s="16" t="n"/>
+      <c r="H31" s="17" t="n"/>
       <c r="I31" s="11" t="n"/>
-      <c r="J31" s="15" t="n"/>
+      <c r="J31" s="16" t="n"/>
       <c r="K31" s="11" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="n"/>
-      <c r="B32" s="13" t="n"/>
-      <c r="C32" s="14" t="n"/>
-      <c r="D32" s="14" t="n"/>
+      <c r="A32" s="17" t="n"/>
+      <c r="B32" s="17" t="n"/>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
       <c r="E32" s="11" t="n"/>
       <c r="F32" s="11" t="n"/>
-      <c r="G32" s="15" t="n"/>
-      <c r="H32" s="13" t="n"/>
+      <c r="G32" s="16" t="n"/>
+      <c r="H32" s="17" t="n"/>
       <c r="I32" s="11" t="n"/>
-      <c r="J32" s="15" t="n"/>
+      <c r="J32" s="16" t="n"/>
       <c r="K32" s="11" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="n"/>
-      <c r="B33" s="13" t="n"/>
-      <c r="C33" s="14" t="n"/>
-      <c r="D33" s="14" t="n"/>
+      <c r="A33" s="17" t="n"/>
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="15" t="n"/>
       <c r="E33" s="11" t="n"/>
       <c r="F33" s="11" t="n"/>
-      <c r="G33" s="15" t="n"/>
-      <c r="H33" s="13" t="n"/>
+      <c r="G33" s="16" t="n"/>
+      <c r="H33" s="17" t="n"/>
       <c r="I33" s="11" t="n"/>
-      <c r="J33" s="15" t="n"/>
+      <c r="J33" s="16" t="n"/>
       <c r="K33" s="11" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="n"/>
-      <c r="B34" s="13" t="n"/>
-      <c r="C34" s="14" t="n"/>
-      <c r="D34" s="14" t="n"/>
+      <c r="A34" s="17" t="n"/>
+      <c r="B34" s="17" t="n"/>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="n"/>
       <c r="E34" s="11" t="n"/>
       <c r="F34" s="11" t="n"/>
-      <c r="G34" s="15" t="n"/>
-      <c r="H34" s="13" t="n"/>
+      <c r="G34" s="16" t="n"/>
+      <c r="H34" s="17" t="n"/>
       <c r="I34" s="11" t="n"/>
-      <c r="J34" s="15" t="n"/>
+      <c r="J34" s="16" t="n"/>
       <c r="K34" s="11" t="n"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use short event codes (CN2026 etc.) in template and dashboard
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HBvLiZRp3wB8j46GxyLbc4
</commit_message>
<xml_diff>
--- a/template/MCE-monthly-data-template.xlsx
+++ b/template/MCE-monthly-data-template.xlsx
@@ -234,7 +234,7 @@
   <commentList>
     <comment ref="A4" authorId="0" shapeId="0">
       <text>
-        <t>The event's code in PheedLoop (in the event URL or Event Settings)</t>
+        <t>Short code such as CN2026, linked to its PheedLoop event. For a new event, ask Claude to add a code or use its PheedLoop code (starts with EVE).</t>
       </text>
     </comment>
     <comment ref="B4" authorId="0" shapeId="0">
@@ -259,7 +259,7 @@
     </comment>
     <comment ref="H4" authorId="0" shapeId="0">
       <text>
-        <t>Optional, links this event to last year's for comparison</t>
+        <t>Optional, e.g. CN2025, to compare with last year's event</t>
       </text>
     </comment>
     <comment ref="I4" authorId="0" shapeId="0">
@@ -3050,7 +3050,7 @@
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>EVELJKYPBEJHY</t>
+          <t>CN2026</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
@@ -3073,7 +3073,7 @@
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>EVEBXNZTBEUUH</t>
+          <t>SAIC2026</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
@@ -3096,7 +3096,7 @@
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>EVEAQFBMZWRVS</t>
+          <t>YPADEC2026</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
@@ -3119,7 +3119,7 @@
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>EVEMZGBXYIECC</t>
+          <t>MANL2026</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
@@ -3142,7 +3142,7 @@
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>EVEHLZEOSVFCO</t>
+          <t>CAIC2027</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
@@ -3165,7 +3165,7 @@
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>EVERJBXTUBTOJ</t>
+          <t>CCIFMON2026</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
@@ -3188,7 +3188,7 @@
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>EVEYTSAMYGMAZ</t>
+          <t>QCGOLF2026</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
@@ -3211,7 +3211,7 @@
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>EVESVVXRAORUS</t>
+          <t>ABGOLF2026</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
@@ -3234,7 +3234,7 @@
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>EVEEACRKBFWWT</t>
+          <t>MBGOLF2026</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Upload checks, engaged-session quality metrics, email fatigue chart, yearly targets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HBvLiZRp3wB8j46GxyLbc4
</commit_message>
<xml_diff>
--- a/template/MCE-monthly-data-template.xlsx
+++ b/template/MCE-monthly-data-template.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targets" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,9 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="$#,##0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -129,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,6 +153,8 @@
     <xf numFmtId="164" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -570,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -732,55 +737,51 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Targets</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Yearly goals for website, email, social and events. Fill them in once; re-upload only when they change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Example (format only; not uploaded)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Breakdown</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Website (GA4)</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Sessions</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr"/>
-      <c r="D21" s="8" t="n">
-        <v>18420</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Sessions by channel (GA4)</t>
+          <t>Website (GA4)</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -788,32 +789,48 @@
           <t>Sessions</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
+      <c r="C22" s="7" t="inlineStr"/>
       <c r="D22" s="8" t="n">
-        <v>3130</v>
+        <v>18420</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
+          <t>Sessions by channel (GA4)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Sessions</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>3130</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
           <t>Social</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Engagements</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="D23" s="8" t="n">
+      <c r="D24" s="8" t="n">
         <v>1482</v>
       </c>
     </row>
@@ -3531,4 +3548,653 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col hidden="1" width="12" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="12" customWidth="1" min="7" max="7"/>
+    <col hidden="1" width="22" customWidth="1" min="8" max="8"/>
+    <col hidden="1" width="12" customWidth="1" min="9" max="9"/>
+    <col hidden="1" width="8" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="8" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Targets</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Yearly goals for each stream. Fill in only the targets you want; blank cells are skipped. The dashboard shows whether each one is on pace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Percentages: type them with a % sign (e.g. 25%). Event targets count events held during the year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Stream</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>How it's measured</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>2026 target</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>2027 target</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>stream</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>metric_key</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>dimension</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>better</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Engaged website sessions</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Total for the year (GA4 engaged sessions)</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>ga4</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>engaged_sessions</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr"/>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>higher</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Website key events (conversions)</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Total for the year</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>ga4</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>key_events</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr"/>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>higher</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Website engagement rate</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Engaged sessions ÷ sessions, year to date</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>ga4</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>engagement_rate</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr"/>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>higher</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Communications</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Email unique open rate</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Unique opens ÷ delivered, year to date</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="n"/>
+      <c r="E8" s="18" t="n"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>communications</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>insightly</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>open_rate</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr"/>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>higher</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Communications</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Email unique click rate</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Unique clicks ÷ delivered, year to date</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>communications</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>insightly</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>click_rate</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr"/>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>higher</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Communications</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Opt-outs per broad send</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Main-list opt-outs ÷ broad sends (lower is better)</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>communications</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>insightly</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>opt_outs_per_broad_send</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr"/>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>dec</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Communications</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Broad sends to a member per month</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Monthly average (lower is better; the audit cap is about 9)</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="n"/>
+      <c r="E11" s="19" t="n"/>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>communications</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>insightly</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>broad_sends_avg</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr"/>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>dec</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Communications</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>LinkedIn followers</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Followers at year end</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>communications</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>social</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>followers</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>higher</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Communications</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Social engagements, all platforms</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Total for the year</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>communications</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>social</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>engagements_all</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr"/>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>higher</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Event registrations (events held)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Registrations for events held during the year</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>pheedloop</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>registrations_held</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr"/>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>higher</t>
+        </is>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Event attendance (checked in)</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Checked-in attendees for events held during the year</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>pheedloop</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>attendance_held</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr"/>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>higher</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Event revenue</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Revenue for events held during the year</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>pheedloop</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>revenue_held</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr"/>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>higher</t>
+        </is>
+      </c>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>money</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Enter yearly targets on the upload page; remove Targets tab from template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HBvLiZRp3wB8j46GxyLbc4
</commit_message>
<xml_diff>
--- a/template/MCE-monthly-data-template.xlsx
+++ b/template/MCE-monthly-data-template.xlsx
@@ -11,7 +11,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targets" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,11 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="$#,##0"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -132,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,8 +150,6 @@
     <xf numFmtId="164" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -575,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -737,51 +732,55 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Targets</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Yearly goals for website, email, social and events. Fill them in once; re-upload only when they change.</t>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Example (format only; not uploaded)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Example (format only; not uploaded)</t>
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Breakdown</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Breakdown</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Website (GA4)</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Sessions</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr"/>
+      <c r="D21" s="8" t="n">
+        <v>18420</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Website (GA4)</t>
+          <t>Sessions by channel (GA4)</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -789,48 +788,32 @@
           <t>Sessions</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr"/>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
       <c r="D22" s="8" t="n">
-        <v>18420</v>
+        <v>3130</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Sessions by channel (GA4)</t>
+          <t>Social</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Sessions</t>
+          <t>Engagements</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>3130</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>Social</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Engagements</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="n">
         <v>1482</v>
       </c>
     </row>
@@ -3548,653 +3531,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col hidden="1" width="12" customWidth="1" min="6" max="6"/>
-    <col hidden="1" width="12" customWidth="1" min="7" max="7"/>
-    <col hidden="1" width="22" customWidth="1" min="8" max="8"/>
-    <col hidden="1" width="12" customWidth="1" min="9" max="9"/>
-    <col hidden="1" width="8" customWidth="1" min="10" max="10"/>
-    <col hidden="1" width="8" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Targets</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Yearly goals for each stream. Fill in only the targets you want; blank cells are skipped. The dashboard shows whether each one is on pace.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Percentages: type them with a % sign (e.g. 25%). Event targets count events held during the year.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Stream</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Measure</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>How it's measured</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>2026 target</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>2027 target</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
-        <is>
-          <t>stream</t>
-        </is>
-      </c>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="H4" s="12" t="inlineStr">
-        <is>
-          <t>metric_key</t>
-        </is>
-      </c>
-      <c r="I4" s="12" t="inlineStr">
-        <is>
-          <t>dimension</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="inlineStr">
-        <is>
-          <t>better</t>
-        </is>
-      </c>
-      <c r="K4" s="12" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Engaged website sessions</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Total for the year (GA4 engaged sessions)</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="n"/>
-      <c r="E5" s="11" t="n"/>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>marketing</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>ga4</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>engaged_sessions</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr"/>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>higher</t>
-        </is>
-      </c>
-      <c r="K5" s="7" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Website key events (conversions)</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Total for the year</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="n"/>
-      <c r="E6" s="11" t="n"/>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>marketing</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>ga4</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>key_events</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr"/>
-      <c r="J6" s="7" t="inlineStr">
-        <is>
-          <t>higher</t>
-        </is>
-      </c>
-      <c r="K6" s="7" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Website engagement rate</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Engaged sessions ÷ sessions, year to date</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="n"/>
-      <c r="E7" s="18" t="n"/>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>marketing</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>ga4</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>engagement_rate</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr"/>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>higher</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>pct</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Communications</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Email unique open rate</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Unique opens ÷ delivered, year to date</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="n"/>
-      <c r="E8" s="18" t="n"/>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>communications</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>insightly</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>open_rate</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr"/>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>higher</t>
-        </is>
-      </c>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>pct</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Communications</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Email unique click rate</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Unique clicks ÷ delivered, year to date</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="n"/>
-      <c r="E9" s="18" t="n"/>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>communications</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>insightly</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>click_rate</t>
-        </is>
-      </c>
-      <c r="I9" s="7" t="inlineStr"/>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>higher</t>
-        </is>
-      </c>
-      <c r="K9" s="7" t="inlineStr">
-        <is>
-          <t>pct</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Communications</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Opt-outs per broad send</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Main-list opt-outs ÷ broad sends (lower is better)</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="19" t="n"/>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>communications</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>insightly</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>opt_outs_per_broad_send</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr"/>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>lower</t>
-        </is>
-      </c>
-      <c r="K10" s="7" t="inlineStr">
-        <is>
-          <t>dec</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Communications</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Broad sends to a member per month</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Monthly average (lower is better; the audit cap is about 9)</t>
-        </is>
-      </c>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="19" t="n"/>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>communications</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>insightly</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>broad_sends_avg</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr"/>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>lower</t>
-        </is>
-      </c>
-      <c r="K11" s="7" t="inlineStr">
-        <is>
-          <t>dec</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Communications</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>LinkedIn followers</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Followers at year end</t>
-        </is>
-      </c>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>communications</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>social</t>
-        </is>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>followers</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="J12" s="7" t="inlineStr">
-        <is>
-          <t>higher</t>
-        </is>
-      </c>
-      <c r="K12" s="7" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Communications</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Social engagements, all platforms</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Total for the year</t>
-        </is>
-      </c>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>communications</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>social</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>engagements_all</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="inlineStr"/>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>higher</t>
-        </is>
-      </c>
-      <c r="K13" s="7" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Event registrations (events held)</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Registrations for events held during the year</t>
-        </is>
-      </c>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>engagement</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>pheedloop</t>
-        </is>
-      </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>registrations_held</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="inlineStr"/>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>higher</t>
-        </is>
-      </c>
-      <c r="K14" s="7" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Event attendance (checked in)</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Checked-in attendees for events held during the year</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>engagement</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>pheedloop</t>
-        </is>
-      </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>attendance_held</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="inlineStr"/>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>higher</t>
-        </is>
-      </c>
-      <c r="K15" s="7" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Event revenue</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Revenue for events held during the year</t>
-        </is>
-      </c>
-      <c r="D16" s="16" t="n"/>
-      <c r="E16" s="16" t="n"/>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>engagement</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>pheedloop</t>
-        </is>
-      </c>
-      <c r="H16" s="7" t="inlineStr">
-        <is>
-          <t>revenue_held</t>
-        </is>
-      </c>
-      <c r="I16" s="7" t="inlineStr"/>
-      <c r="J16" s="7" t="inlineStr">
-        <is>
-          <t>higher</t>
-        </is>
-      </c>
-      <c r="K16" s="7" t="inlineStr">
-        <is>
-          <t>money</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Every-event-this-year table; short codes for CAIC2026, GRV2026, BCGOLF2026 and 2025 events; template prefill
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HBvLiZRp3wB8j46GxyLbc4
</commit_message>
<xml_diff>
--- a/template/MCE-monthly-data-template.xlsx
+++ b/template/MCE-monthly-data-template.xlsx
@@ -3050,16 +3050,16 @@
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>CN2026</t>
+          <t>CAIC2026</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Canada Night 2026</t>
+          <t>Canadian Auto Care Industry Conference 2026</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>46329</v>
+        <v>46092</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="11" t="n"/>
@@ -3073,16 +3073,16 @@
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>SAIC2026</t>
+          <t>GRV2026</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Student Automotive Innovation Challenge 2026</t>
+          <t>Le Grand Rendez-Vous (Québec Division) 2026</t>
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>46344</v>
+        <v>46170</v>
       </c>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="11" t="n"/>
@@ -3096,16 +3096,16 @@
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>YPADEC2026</t>
+          <t>BCGOLF2026</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>YPA Community Learning and Leadership Social 2026</t>
+          <t>AIA Canada British Columbia Division Golf Tournament 2026</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>46359</v>
+        <v>46243</v>
       </c>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="11" t="n"/>
@@ -3119,16 +3119,16 @@
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>MANL2026</t>
+          <t>CN2026</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>AIA Canada Manitoba Division Holiday Luncheon 2026</t>
+          <t>Canada Night 2026</t>
         </is>
       </c>
       <c r="C8" s="14" t="n">
-        <v>46367</v>
+        <v>46329</v>
       </c>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="11" t="n"/>
@@ -3142,16 +3142,16 @@
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>CAIC2027</t>
+          <t>SAIC2026</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>CAIC 2027</t>
+          <t>Student Automotive Innovation Challenge 2026</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>46476</v>
+        <v>46344</v>
       </c>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="11" t="n"/>
@@ -3165,16 +3165,16 @@
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>CCIFMON2026</t>
+          <t>YPADEC2026</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>CCIF Montreal 2026</t>
+          <t>YPA Community Learning and Leadership Social 2026</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>46281</v>
+        <v>46359</v>
       </c>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="11" t="n"/>
@@ -3188,16 +3188,16 @@
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>QCGOLF2026</t>
+          <t>MANL2026</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Tournoi de golf de la division du Québec de l'AIA Canada 2026</t>
+          <t>AIA Canada Manitoba Division Holiday Luncheon 2026</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>46261</v>
+        <v>46367</v>
       </c>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="11" t="n"/>
@@ -3211,16 +3211,16 @@
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>ABGOLF2026</t>
+          <t>CAIC2027</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>AIA Canada Alberta Division golf tournament 2026</t>
+          <t>CAIC 2027</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>46266</v>
+        <v>46476</v>
       </c>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="11" t="n"/>
@@ -3234,16 +3234,16 @@
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>MBGOLF2026</t>
+          <t>CCIFMON2026</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>AIA Canada Manitoba Division golf tournament 2026</t>
+          <t>CCIF Montreal 2026</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>46268</v>
+        <v>46281</v>
       </c>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="11" t="n"/>
@@ -3255,9 +3255,19 @@
       <c r="K13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="n"/>
-      <c r="B14" s="17" t="n"/>
-      <c r="C14" s="15" t="n"/>
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>QCGOLF2026</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Tournoi de golf de la division du Québec de l'AIA Canada 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>46261</v>
+      </c>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="11" t="n"/>
       <c r="F14" s="11" t="n"/>
@@ -3268,9 +3278,19 @@
       <c r="K14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="n"/>
-      <c r="B15" s="17" t="n"/>
-      <c r="C15" s="15" t="n"/>
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>ABGOLF2026</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>AIA Canada Alberta Division golf tournament 2026</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>46266</v>
+      </c>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="11" t="n"/>
       <c r="F15" s="11" t="n"/>
@@ -3281,9 +3301,19 @@
       <c r="K15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="n"/>
-      <c r="B16" s="17" t="n"/>
-      <c r="C16" s="15" t="n"/>
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>MBGOLF2026</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>AIA Canada Manitoba Division golf tournament 2026</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>46268</v>
+      </c>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="11" t="n"/>
       <c r="F16" s="11" t="n"/>

</xml_diff>